<commit_message>
Add Parts Desk desktop app; make workbook formulas Google Sheets-safe
PartsDesk.html is a single-file offline app (dashboard, RFQ log, quote
calculator, suppliers, customers, settings, backup/restore). Workbook
dashboard formulas no longer rely on array constants, which Google
Sheets evaluated as zero for 'Profit in play'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015afof7uAjH2dPBJuyUD5QL
</commit_message>
<xml_diff>
--- a/sunsystems-broker/SunSystems_Parts_Desk.xlsx
+++ b/sunsystems-broker/SunSystems_Parts_Desk.xlsx
@@ -1857,11 +1857,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="34523354"/>
-        <c:axId val="40302229"/>
+        <c:axId val="89267892"/>
+        <c:axId val="38478474"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34523354"/>
+        <c:axId val="89267892"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1893,7 +1893,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40302229"/>
+        <c:crossAx val="38478474"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1901,7 +1901,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40302229"/>
+        <c:axId val="38478474"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1977,7 +1977,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34523354"/>
+        <c:crossAx val="89267892"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2642,7 +2642,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="str">
         <f aca="true">"As of "&amp;TEXT(TODAY(),"mmm d, yyyy")</f>
-        <v>As of Oct 13, 2026</v>
+        <v>As of Oct 14, 2026</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -2728,7 +2728,7 @@
         <v>80</v>
       </c>
       <c r="B7" s="13" t="n">
-        <f aca="false">SUMPRODUCT(SUMIFS('RFQ Log'!$P$5:$P$304,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped"}))</f>
+        <f aca="false">SUMIFS('RFQ Log'!$P$5:$P$304,'RFQ Log'!$R$5:$R$304,"Won")+SUMIFS('RFQ Log'!$P$5:$P$304,'RFQ Log'!$R$5:$R$304,"Ordered")+SUMIFS('RFQ Log'!$P$5:$P$304,'RFQ Log'!$R$5:$R$304,"Shipped")</f>
         <v>375.5</v>
       </c>
       <c r="C7" s="1"/>
@@ -2846,7 +2846,7 @@
         <v>91</v>
       </c>
       <c r="B13" s="17" t="n">
-        <f aca="false">IFERROR(SUMPRODUCT(COUNTIF('RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"}))/(SUMPRODUCT(COUNTIF('RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"}))+COUNTIF('RFQ Log'!$R$5:$R$304,"Lost")),0)</f>
+        <f aca="false">IFERROR((COUNTIF('RFQ Log'!$R$5:$R$304,"Won")+COUNTIF('RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIF('RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIF('RFQ Log'!$R$5:$R$304,"Paid"))/((COUNTIF('RFQ Log'!$R$5:$R$304,"Won")+COUNTIF('RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIF('RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIF('RFQ Log'!$R$5:$R$304,"Paid"))+COUNTIF('RFQ Log'!$R$5:$R$304,"Lost")),0)</f>
         <v>1</v>
       </c>
       <c r="C13" s="1"/>
@@ -2859,7 +2859,7 @@
         <v>92</v>
       </c>
       <c r="B14" s="37" t="n">
-        <f aca="false">SUMPRODUCT(COUNTIF('RFQ Log'!$R$5:$R$304,{"New","Sourcing","Quoted"}))</f>
+        <f aca="false">COUNTIF('RFQ Log'!$R$5:$R$304,"New")+COUNTIF('RFQ Log'!$R$5:$R$304,"Sourcing")+COUNTIF('RFQ Log'!$R$5:$R$304,"Quoted")</f>
         <v>1</v>
       </c>
       <c r="C14" s="1"/>
@@ -2872,7 +2872,7 @@
         <v>93</v>
       </c>
       <c r="B15" s="37" t="n">
-        <f aca="true">SUMPRODUCT(('RFQ Log'!$S$5:$S$304&lt;&gt;"")*('RFQ Log'!$S$5:$S$304&lt;=TODAY())*(('RFQ Log'!$R$5:$R$304="New")+('RFQ Log'!$R$5:$R$304="Sourcing")+('RFQ Log'!$R$5:$R$304="Quoted")))</f>
+        <f aca="true">COUNTIFS('RFQ Log'!$S$5:$S$304,"&lt;="&amp;TODAY(),'RFQ Log'!$R$5:$R$304,"New")+COUNTIFS('RFQ Log'!$S$5:$S$304,"&lt;="&amp;TODAY(),'RFQ Log'!$R$5:$R$304,"Sourcing")+COUNTIFS('RFQ Log'!$S$5:$S$304,"&lt;="&amp;TODAY(),'RFQ Log'!$R$5:$R$304,"Quoted")</f>
         <v>1</v>
       </c>
       <c r="C15" s="1"/>
@@ -3505,7 +3505,7 @@
         <v>140</v>
       </c>
       <c r="B6" s="53" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="B7" s="54" t="n">
         <f aca="false">B6+Settings!$B$7</f>
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -4446,7 +4446,7 @@
         <v>Q-001</v>
       </c>
       <c r="B5" s="53" t="n">
-        <v>46268</v>
+        <v>46269</v>
       </c>
       <c r="C5" s="52" t="s">
         <v>137</v>
@@ -4461,7 +4461,7 @@
         <v>8</v>
       </c>
       <c r="G5" s="53" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="H5" s="52" t="s">
         <v>199</v>
@@ -4509,7 +4509,7 @@
         <v/>
       </c>
       <c r="U5" s="53" t="n">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="V5" s="66" t="s">
         <v>200</v>
@@ -4521,7 +4521,7 @@
         <v>Q-002</v>
       </c>
       <c r="B6" s="53" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="C6" s="52" t="s">
         <v>201</v>
@@ -4536,7 +4536,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="53" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="H6" s="52" t="s">
         <v>204</v>
@@ -4596,7 +4596,7 @@
         <v>Q-003</v>
       </c>
       <c r="B7" s="53" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="C7" s="52" t="s">
         <v>137</v>
@@ -4611,7 +4611,7 @@
         <v>2</v>
       </c>
       <c r="G7" s="53" t="n">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="H7" s="52" t="s">
         <v>199</v>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="S7" s="65" t="n">
         <f aca="false">IF(OR(B7="",R7="Paid",R7="Lost",R7="Shipped"),"",B7+Settings!$B$8)</f>
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="T7" s="10" t="n">
         <f aca="true">IF(OR(B7="",R7="Paid",R7="Lost"),"",TODAY()-B7)</f>
@@ -23330,7 +23330,7 @@
         <v>2</v>
       </c>
       <c r="H5" s="67" t="n">
-        <f aca="false">IF(A5="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A5,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A5="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A5,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A5,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A5,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A5,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v>1</v>
       </c>
       <c r="I5" s="69" t="n">
@@ -23373,7 +23373,7 @@
         <v>1</v>
       </c>
       <c r="H6" s="67" t="n">
-        <f aca="false">IF(A6="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A6,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A6="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A6,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A6,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A6,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A6,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v>1</v>
       </c>
       <c r="I6" s="69" t="n">
@@ -23404,7 +23404,7 @@
         <v/>
       </c>
       <c r="H7" s="67" t="str">
-        <f aca="false">IF(A7="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A7,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A7="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A7,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A7,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A7,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A7,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I7" s="69" t="str">
@@ -23433,7 +23433,7 @@
         <v/>
       </c>
       <c r="H8" s="67" t="str">
-        <f aca="false">IF(A8="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A8,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A8="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A8,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A8,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A8,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A8,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I8" s="69" t="str">
@@ -23462,7 +23462,7 @@
         <v/>
       </c>
       <c r="H9" s="67" t="str">
-        <f aca="false">IF(A9="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A9,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A9="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A9,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A9,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A9,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A9,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I9" s="69" t="str">
@@ -23491,7 +23491,7 @@
         <v/>
       </c>
       <c r="H10" s="67" t="str">
-        <f aca="false">IF(A10="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A10,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A10="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A10,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A10,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A10,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A10,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I10" s="69" t="str">
@@ -23520,7 +23520,7 @@
         <v/>
       </c>
       <c r="H11" s="67" t="str">
-        <f aca="false">IF(A11="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A11,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A11="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A11,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A11,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A11,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A11,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I11" s="69" t="str">
@@ -23549,7 +23549,7 @@
         <v/>
       </c>
       <c r="H12" s="67" t="str">
-        <f aca="false">IF(A12="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A12,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A12="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A12,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A12,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A12,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A12,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I12" s="69" t="str">
@@ -23578,7 +23578,7 @@
         <v/>
       </c>
       <c r="H13" s="67" t="str">
-        <f aca="false">IF(A13="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A13,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A13="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A13,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A13,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A13,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A13,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I13" s="69" t="str">
@@ -23607,7 +23607,7 @@
         <v/>
       </c>
       <c r="H14" s="67" t="str">
-        <f aca="false">IF(A14="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A14,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A14="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A14,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A14,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A14,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A14,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I14" s="69" t="str">
@@ -23636,7 +23636,7 @@
         <v/>
       </c>
       <c r="H15" s="67" t="str">
-        <f aca="false">IF(A15="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A15,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A15="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A15,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A15,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A15,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A15,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I15" s="69" t="str">
@@ -23665,7 +23665,7 @@
         <v/>
       </c>
       <c r="H16" s="67" t="str">
-        <f aca="false">IF(A16="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A16,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A16="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A16,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A16,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A16,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A16,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I16" s="69" t="str">
@@ -23694,7 +23694,7 @@
         <v/>
       </c>
       <c r="H17" s="67" t="str">
-        <f aca="false">IF(A17="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A17,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A17="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A17,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A17,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A17,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A17,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I17" s="69" t="str">
@@ -23723,7 +23723,7 @@
         <v/>
       </c>
       <c r="H18" s="67" t="str">
-        <f aca="false">IF(A18="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A18,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A18="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A18,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A18,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A18,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A18,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I18" s="69" t="str">
@@ -23752,7 +23752,7 @@
         <v/>
       </c>
       <c r="H19" s="67" t="str">
-        <f aca="false">IF(A19="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A19,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A19="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A19,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A19,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A19,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A19,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I19" s="69" t="str">
@@ -23781,7 +23781,7 @@
         <v/>
       </c>
       <c r="H20" s="67" t="str">
-        <f aca="false">IF(A20="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A20,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A20="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A20,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A20,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A20,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A20,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I20" s="69" t="str">
@@ -23810,7 +23810,7 @@
         <v/>
       </c>
       <c r="H21" s="67" t="str">
-        <f aca="false">IF(A21="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A21,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A21="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A21,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A21,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A21,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A21,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I21" s="69" t="str">
@@ -23839,7 +23839,7 @@
         <v/>
       </c>
       <c r="H22" s="67" t="str">
-        <f aca="false">IF(A22="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A22,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A22="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A22,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A22,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A22,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A22,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I22" s="69" t="str">
@@ -23868,7 +23868,7 @@
         <v/>
       </c>
       <c r="H23" s="67" t="str">
-        <f aca="false">IF(A23="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A23,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A23="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A23,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A23,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A23,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A23,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I23" s="69" t="str">
@@ -23897,7 +23897,7 @@
         <v/>
       </c>
       <c r="H24" s="67" t="str">
-        <f aca="false">IF(A24="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A24,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A24="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A24,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A24,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A24,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A24,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I24" s="69" t="str">
@@ -23926,7 +23926,7 @@
         <v/>
       </c>
       <c r="H25" s="67" t="str">
-        <f aca="false">IF(A25="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A25,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A25="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A25,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A25,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A25,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A25,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I25" s="69" t="str">
@@ -23955,7 +23955,7 @@
         <v/>
       </c>
       <c r="H26" s="67" t="str">
-        <f aca="false">IF(A26="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A26,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A26="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A26,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A26,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A26,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A26,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I26" s="69" t="str">
@@ -23984,7 +23984,7 @@
         <v/>
       </c>
       <c r="H27" s="67" t="str">
-        <f aca="false">IF(A27="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A27,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A27="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A27,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A27,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A27,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A27,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I27" s="69" t="str">
@@ -24013,7 +24013,7 @@
         <v/>
       </c>
       <c r="H28" s="67" t="str">
-        <f aca="false">IF(A28="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A28,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A28="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A28,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A28,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A28,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A28,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I28" s="69" t="str">
@@ -24042,7 +24042,7 @@
         <v/>
       </c>
       <c r="H29" s="67" t="str">
-        <f aca="false">IF(A29="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A29,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A29="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A29,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A29,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A29,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A29,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I29" s="69" t="str">
@@ -24071,7 +24071,7 @@
         <v/>
       </c>
       <c r="H30" s="67" t="str">
-        <f aca="false">IF(A30="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A30,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A30="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A30,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A30,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A30,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A30,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I30" s="69" t="str">
@@ -24100,7 +24100,7 @@
         <v/>
       </c>
       <c r="H31" s="67" t="str">
-        <f aca="false">IF(A31="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A31,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A31="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A31,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A31,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A31,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A31,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I31" s="69" t="str">
@@ -24129,7 +24129,7 @@
         <v/>
       </c>
       <c r="H32" s="67" t="str">
-        <f aca="false">IF(A32="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A32,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A32="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A32,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A32,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A32,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A32,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I32" s="69" t="str">
@@ -24158,7 +24158,7 @@
         <v/>
       </c>
       <c r="H33" s="67" t="str">
-        <f aca="false">IF(A33="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A33,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A33="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A33,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A33,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A33,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A33,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I33" s="69" t="str">
@@ -24187,7 +24187,7 @@
         <v/>
       </c>
       <c r="H34" s="67" t="str">
-        <f aca="false">IF(A34="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A34,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A34="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A34,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A34,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A34,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A34,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I34" s="69" t="str">
@@ -24216,7 +24216,7 @@
         <v/>
       </c>
       <c r="H35" s="67" t="str">
-        <f aca="false">IF(A35="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A35,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A35="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A35,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A35,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A35,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A35,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I35" s="69" t="str">
@@ -24245,7 +24245,7 @@
         <v/>
       </c>
       <c r="H36" s="67" t="str">
-        <f aca="false">IF(A36="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A36,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A36="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A36,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A36,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A36,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A36,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I36" s="69" t="str">
@@ -24274,7 +24274,7 @@
         <v/>
       </c>
       <c r="H37" s="67" t="str">
-        <f aca="false">IF(A37="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A37,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A37="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A37,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A37,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A37,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A37,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I37" s="69" t="str">
@@ -24303,7 +24303,7 @@
         <v/>
       </c>
       <c r="H38" s="67" t="str">
-        <f aca="false">IF(A38="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A38,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A38="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A38,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A38,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A38,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A38,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I38" s="69" t="str">
@@ -24332,7 +24332,7 @@
         <v/>
       </c>
       <c r="H39" s="67" t="str">
-        <f aca="false">IF(A39="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A39,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A39="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A39,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A39,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A39,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A39,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I39" s="69" t="str">
@@ -24361,7 +24361,7 @@
         <v/>
       </c>
       <c r="H40" s="67" t="str">
-        <f aca="false">IF(A40="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A40,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A40="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A40,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A40,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A40,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A40,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I40" s="69" t="str">
@@ -24390,7 +24390,7 @@
         <v/>
       </c>
       <c r="H41" s="67" t="str">
-        <f aca="false">IF(A41="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A41,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A41="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A41,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A41,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A41,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A41,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I41" s="69" t="str">
@@ -24419,7 +24419,7 @@
         <v/>
       </c>
       <c r="H42" s="67" t="str">
-        <f aca="false">IF(A42="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A42,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A42="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A42,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A42,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A42,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A42,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I42" s="69" t="str">
@@ -24448,7 +24448,7 @@
         <v/>
       </c>
       <c r="H43" s="67" t="str">
-        <f aca="false">IF(A43="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A43,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A43="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A43,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A43,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A43,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A43,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I43" s="69" t="str">
@@ -24477,7 +24477,7 @@
         <v/>
       </c>
       <c r="H44" s="67" t="str">
-        <f aca="false">IF(A44="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A44,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A44="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A44,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A44,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A44,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A44,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I44" s="69" t="str">
@@ -24506,7 +24506,7 @@
         <v/>
       </c>
       <c r="H45" s="67" t="str">
-        <f aca="false">IF(A45="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A45,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A45="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A45,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A45,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A45,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A45,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I45" s="69" t="str">
@@ -24535,7 +24535,7 @@
         <v/>
       </c>
       <c r="H46" s="67" t="str">
-        <f aca="false">IF(A46="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A46,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A46="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A46,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A46,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A46,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A46,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I46" s="69" t="str">
@@ -24564,7 +24564,7 @@
         <v/>
       </c>
       <c r="H47" s="67" t="str">
-        <f aca="false">IF(A47="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A47,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A47="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A47,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A47,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A47,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A47,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I47" s="69" t="str">
@@ -24593,7 +24593,7 @@
         <v/>
       </c>
       <c r="H48" s="67" t="str">
-        <f aca="false">IF(A48="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A48,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A48="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A48,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A48,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A48,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A48,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I48" s="69" t="str">
@@ -24622,7 +24622,7 @@
         <v/>
       </c>
       <c r="H49" s="67" t="str">
-        <f aca="false">IF(A49="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A49,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A49="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A49,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A49,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A49,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A49,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I49" s="69" t="str">
@@ -24651,7 +24651,7 @@
         <v/>
       </c>
       <c r="H50" s="67" t="str">
-        <f aca="false">IF(A50="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A50,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A50="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A50,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A50,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A50,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A50,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I50" s="69" t="str">
@@ -24680,7 +24680,7 @@
         <v/>
       </c>
       <c r="H51" s="67" t="str">
-        <f aca="false">IF(A51="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A51,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A51="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A51,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A51,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A51,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A51,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I51" s="69" t="str">
@@ -24709,7 +24709,7 @@
         <v/>
       </c>
       <c r="H52" s="67" t="str">
-        <f aca="false">IF(A52="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A52,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A52="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A52,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A52,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A52,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A52,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I52" s="69" t="str">
@@ -24738,7 +24738,7 @@
         <v/>
       </c>
       <c r="H53" s="67" t="str">
-        <f aca="false">IF(A53="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A53,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A53="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A53,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A53,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A53,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A53,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I53" s="69" t="str">
@@ -24767,7 +24767,7 @@
         <v/>
       </c>
       <c r="H54" s="67" t="str">
-        <f aca="false">IF(A54="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A54,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A54="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A54,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A54,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A54,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A54,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I54" s="69" t="str">
@@ -24796,7 +24796,7 @@
         <v/>
       </c>
       <c r="H55" s="67" t="str">
-        <f aca="false">IF(A55="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A55,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A55="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A55,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A55,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A55,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A55,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I55" s="69" t="str">
@@ -24825,7 +24825,7 @@
         <v/>
       </c>
       <c r="H56" s="67" t="str">
-        <f aca="false">IF(A56="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A56,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A56="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A56,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A56,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A56,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A56,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I56" s="69" t="str">
@@ -24854,7 +24854,7 @@
         <v/>
       </c>
       <c r="H57" s="67" t="str">
-        <f aca="false">IF(A57="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A57,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A57="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A57,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A57,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A57,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A57,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I57" s="69" t="str">
@@ -24883,7 +24883,7 @@
         <v/>
       </c>
       <c r="H58" s="67" t="str">
-        <f aca="false">IF(A58="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A58,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A58="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A58,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A58,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A58,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A58,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I58" s="69" t="str">
@@ -24912,7 +24912,7 @@
         <v/>
       </c>
       <c r="H59" s="67" t="str">
-        <f aca="false">IF(A59="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A59,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A59="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A59,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A59,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A59,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A59,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I59" s="69" t="str">
@@ -24941,7 +24941,7 @@
         <v/>
       </c>
       <c r="H60" s="67" t="str">
-        <f aca="false">IF(A60="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A60,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A60="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A60,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A60,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A60,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A60,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I60" s="69" t="str">
@@ -24970,7 +24970,7 @@
         <v/>
       </c>
       <c r="H61" s="67" t="str">
-        <f aca="false">IF(A61="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A61,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A61="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A61,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A61,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A61,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A61,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I61" s="69" t="str">
@@ -24999,7 +24999,7 @@
         <v/>
       </c>
       <c r="H62" s="67" t="str">
-        <f aca="false">IF(A62="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A62,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A62="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A62,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A62,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A62,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A62,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I62" s="69" t="str">
@@ -25028,7 +25028,7 @@
         <v/>
       </c>
       <c r="H63" s="67" t="str">
-        <f aca="false">IF(A63="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A63,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A63="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A63,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A63,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A63,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A63,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I63" s="69" t="str">
@@ -25057,7 +25057,7 @@
         <v/>
       </c>
       <c r="H64" s="67" t="str">
-        <f aca="false">IF(A64="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A64,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A64="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A64,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A64,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A64,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A64,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I64" s="69" t="str">
@@ -25086,7 +25086,7 @@
         <v/>
       </c>
       <c r="H65" s="67" t="str">
-        <f aca="false">IF(A65="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A65,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A65="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A65,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A65,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A65,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A65,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I65" s="69" t="str">
@@ -25115,7 +25115,7 @@
         <v/>
       </c>
       <c r="H66" s="67" t="str">
-        <f aca="false">IF(A66="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A66,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A66="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A66,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A66,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A66,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A66,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I66" s="69" t="str">
@@ -25144,7 +25144,7 @@
         <v/>
       </c>
       <c r="H67" s="67" t="str">
-        <f aca="false">IF(A67="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A67,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A67="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A67,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A67,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A67,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A67,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I67" s="69" t="str">
@@ -25173,7 +25173,7 @@
         <v/>
       </c>
       <c r="H68" s="67" t="str">
-        <f aca="false">IF(A68="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A68,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A68="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A68,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A68,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A68,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A68,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I68" s="69" t="str">
@@ -25202,7 +25202,7 @@
         <v/>
       </c>
       <c r="H69" s="67" t="str">
-        <f aca="false">IF(A69="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A69,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A69="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A69,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A69,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A69,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A69,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I69" s="69" t="str">
@@ -25231,7 +25231,7 @@
         <v/>
       </c>
       <c r="H70" s="67" t="str">
-        <f aca="false">IF(A70="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A70,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A70="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A70,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A70,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A70,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A70,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I70" s="69" t="str">
@@ -25260,7 +25260,7 @@
         <v/>
       </c>
       <c r="H71" s="67" t="str">
-        <f aca="false">IF(A71="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A71,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A71="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A71,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A71,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A71,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A71,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I71" s="69" t="str">
@@ -25289,7 +25289,7 @@
         <v/>
       </c>
       <c r="H72" s="67" t="str">
-        <f aca="false">IF(A72="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A72,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A72="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A72,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A72,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A72,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A72,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I72" s="69" t="str">
@@ -25318,7 +25318,7 @@
         <v/>
       </c>
       <c r="H73" s="67" t="str">
-        <f aca="false">IF(A73="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A73,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A73="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A73,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A73,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A73,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A73,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I73" s="69" t="str">
@@ -25347,7 +25347,7 @@
         <v/>
       </c>
       <c r="H74" s="67" t="str">
-        <f aca="false">IF(A74="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A74,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A74="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A74,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A74,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A74,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A74,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I74" s="69" t="str">
@@ -25376,7 +25376,7 @@
         <v/>
       </c>
       <c r="H75" s="67" t="str">
-        <f aca="false">IF(A75="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A75,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A75="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A75,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A75,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A75,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A75,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I75" s="69" t="str">
@@ -25405,7 +25405,7 @@
         <v/>
       </c>
       <c r="H76" s="67" t="str">
-        <f aca="false">IF(A76="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A76,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A76="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A76,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A76,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A76,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A76,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I76" s="69" t="str">
@@ -25434,7 +25434,7 @@
         <v/>
       </c>
       <c r="H77" s="67" t="str">
-        <f aca="false">IF(A77="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A77,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A77="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A77,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A77,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A77,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A77,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I77" s="69" t="str">
@@ -25463,7 +25463,7 @@
         <v/>
       </c>
       <c r="H78" s="67" t="str">
-        <f aca="false">IF(A78="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A78,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A78="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A78,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A78,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A78,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A78,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I78" s="69" t="str">
@@ -25492,7 +25492,7 @@
         <v/>
       </c>
       <c r="H79" s="67" t="str">
-        <f aca="false">IF(A79="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A79,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A79="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A79,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A79,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A79,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A79,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I79" s="69" t="str">
@@ -25521,7 +25521,7 @@
         <v/>
       </c>
       <c r="H80" s="67" t="str">
-        <f aca="false">IF(A80="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A80,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A80="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A80,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A80,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A80,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A80,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I80" s="69" t="str">
@@ -25550,7 +25550,7 @@
         <v/>
       </c>
       <c r="H81" s="67" t="str">
-        <f aca="false">IF(A81="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A81,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A81="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A81,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A81,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A81,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A81,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I81" s="69" t="str">
@@ -25579,7 +25579,7 @@
         <v/>
       </c>
       <c r="H82" s="67" t="str">
-        <f aca="false">IF(A82="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A82,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A82="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A82,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A82,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A82,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A82,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I82" s="69" t="str">
@@ -25608,7 +25608,7 @@
         <v/>
       </c>
       <c r="H83" s="67" t="str">
-        <f aca="false">IF(A83="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A83,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A83="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A83,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A83,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A83,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A83,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I83" s="69" t="str">
@@ -25637,7 +25637,7 @@
         <v/>
       </c>
       <c r="H84" s="67" t="str">
-        <f aca="false">IF(A84="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A84,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A84="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A84,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A84,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A84,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A84,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I84" s="69" t="str">
@@ -25666,7 +25666,7 @@
         <v/>
       </c>
       <c r="H85" s="67" t="str">
-        <f aca="false">IF(A85="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A85,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A85="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A85,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A85,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A85,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A85,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I85" s="69" t="str">
@@ -25695,7 +25695,7 @@
         <v/>
       </c>
       <c r="H86" s="67" t="str">
-        <f aca="false">IF(A86="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A86,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A86="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A86,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A86,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A86,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A86,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I86" s="69" t="str">
@@ -25724,7 +25724,7 @@
         <v/>
       </c>
       <c r="H87" s="67" t="str">
-        <f aca="false">IF(A87="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A87,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A87="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A87,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A87,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A87,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A87,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I87" s="69" t="str">
@@ -25753,7 +25753,7 @@
         <v/>
       </c>
       <c r="H88" s="67" t="str">
-        <f aca="false">IF(A88="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A88,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A88="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A88,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A88,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A88,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A88,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I88" s="69" t="str">
@@ -25782,7 +25782,7 @@
         <v/>
       </c>
       <c r="H89" s="67" t="str">
-        <f aca="false">IF(A89="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A89,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A89="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A89,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A89,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A89,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A89,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I89" s="69" t="str">
@@ -25811,7 +25811,7 @@
         <v/>
       </c>
       <c r="H90" s="67" t="str">
-        <f aca="false">IF(A90="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A90,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A90="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A90,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A90,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A90,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A90,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I90" s="69" t="str">
@@ -25840,7 +25840,7 @@
         <v/>
       </c>
       <c r="H91" s="67" t="str">
-        <f aca="false">IF(A91="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A91,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A91="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A91,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A91,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A91,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A91,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I91" s="69" t="str">
@@ -25869,7 +25869,7 @@
         <v/>
       </c>
       <c r="H92" s="67" t="str">
-        <f aca="false">IF(A92="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A92,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A92="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A92,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A92,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A92,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A92,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I92" s="69" t="str">
@@ -25898,7 +25898,7 @@
         <v/>
       </c>
       <c r="H93" s="67" t="str">
-        <f aca="false">IF(A93="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A93,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A93="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A93,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A93,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A93,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A93,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I93" s="69" t="str">
@@ -25927,7 +25927,7 @@
         <v/>
       </c>
       <c r="H94" s="67" t="str">
-        <f aca="false">IF(A94="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A94,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A94="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A94,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A94,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A94,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A94,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I94" s="69" t="str">
@@ -25956,7 +25956,7 @@
         <v/>
       </c>
       <c r="H95" s="67" t="str">
-        <f aca="false">IF(A95="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A95,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A95="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A95,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A95,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A95,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A95,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I95" s="69" t="str">
@@ -25985,7 +25985,7 @@
         <v/>
       </c>
       <c r="H96" s="67" t="str">
-        <f aca="false">IF(A96="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A96,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A96="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A96,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A96,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A96,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A96,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I96" s="69" t="str">
@@ -26014,7 +26014,7 @@
         <v/>
       </c>
       <c r="H97" s="67" t="str">
-        <f aca="false">IF(A97="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A97,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A97="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A97,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A97,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A97,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A97,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I97" s="69" t="str">
@@ -26043,7 +26043,7 @@
         <v/>
       </c>
       <c r="H98" s="67" t="str">
-        <f aca="false">IF(A98="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A98,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A98="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A98,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A98,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A98,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A98,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I98" s="69" t="str">
@@ -26072,7 +26072,7 @@
         <v/>
       </c>
       <c r="H99" s="67" t="str">
-        <f aca="false">IF(A99="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A99,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A99="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A99,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A99,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A99,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A99,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I99" s="69" t="str">
@@ -26101,7 +26101,7 @@
         <v/>
       </c>
       <c r="H100" s="67" t="str">
-        <f aca="false">IF(A100="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A100,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A100="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A100,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A100,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A100,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A100,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I100" s="69" t="str">
@@ -26130,7 +26130,7 @@
         <v/>
       </c>
       <c r="H101" s="67" t="str">
-        <f aca="false">IF(A101="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A101,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A101="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A101,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A101,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A101,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A101,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I101" s="69" t="str">
@@ -26159,7 +26159,7 @@
         <v/>
       </c>
       <c r="H102" s="67" t="str">
-        <f aca="false">IF(A102="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A102,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A102="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A102,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A102,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A102,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A102,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I102" s="69" t="str">
@@ -26188,7 +26188,7 @@
         <v/>
       </c>
       <c r="H103" s="67" t="str">
-        <f aca="false">IF(A103="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A103,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A103="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A103,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A103,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A103,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A103,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I103" s="69" t="str">
@@ -26217,7 +26217,7 @@
         <v/>
       </c>
       <c r="H104" s="67" t="str">
-        <f aca="false">IF(A104="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A104,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A104="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A104,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A104,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A104,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A104,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I104" s="69" t="str">
@@ -26246,7 +26246,7 @@
         <v/>
       </c>
       <c r="H105" s="67" t="str">
-        <f aca="false">IF(A105="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A105,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A105="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A105,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A105,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A105,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A105,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I105" s="69" t="str">
@@ -26275,7 +26275,7 @@
         <v/>
       </c>
       <c r="H106" s="67" t="str">
-        <f aca="false">IF(A106="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A106,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A106="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A106,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A106,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A106,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A106,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I106" s="69" t="str">
@@ -26304,7 +26304,7 @@
         <v/>
       </c>
       <c r="H107" s="67" t="str">
-        <f aca="false">IF(A107="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A107,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A107="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A107,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A107,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A107,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A107,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I107" s="69" t="str">
@@ -26333,7 +26333,7 @@
         <v/>
       </c>
       <c r="H108" s="67" t="str">
-        <f aca="false">IF(A108="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A108,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A108="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A108,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A108,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A108,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A108,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I108" s="69" t="str">
@@ -26362,7 +26362,7 @@
         <v/>
       </c>
       <c r="H109" s="67" t="str">
-        <f aca="false">IF(A109="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A109,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A109="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A109,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A109,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A109,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A109,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I109" s="69" t="str">
@@ -26391,7 +26391,7 @@
         <v/>
       </c>
       <c r="H110" s="67" t="str">
-        <f aca="false">IF(A110="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A110,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A110="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A110,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A110,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A110,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A110,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I110" s="69" t="str">
@@ -26420,7 +26420,7 @@
         <v/>
       </c>
       <c r="H111" s="67" t="str">
-        <f aca="false">IF(A111="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A111,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A111="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A111,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A111,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A111,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A111,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I111" s="69" t="str">
@@ -26449,7 +26449,7 @@
         <v/>
       </c>
       <c r="H112" s="67" t="str">
-        <f aca="false">IF(A112="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A112,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A112="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A112,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A112,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A112,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A112,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I112" s="69" t="str">
@@ -26478,7 +26478,7 @@
         <v/>
       </c>
       <c r="H113" s="67" t="str">
-        <f aca="false">IF(A113="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A113,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A113="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A113,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A113,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A113,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A113,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I113" s="69" t="str">
@@ -26507,7 +26507,7 @@
         <v/>
       </c>
       <c r="H114" s="67" t="str">
-        <f aca="false">IF(A114="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A114,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A114="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A114,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A114,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A114,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A114,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I114" s="69" t="str">
@@ -26536,7 +26536,7 @@
         <v/>
       </c>
       <c r="H115" s="67" t="str">
-        <f aca="false">IF(A115="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A115,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A115="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A115,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A115,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A115,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A115,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I115" s="69" t="str">
@@ -26565,7 +26565,7 @@
         <v/>
       </c>
       <c r="H116" s="67" t="str">
-        <f aca="false">IF(A116="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A116,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A116="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A116,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A116,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A116,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A116,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I116" s="69" t="str">
@@ -26594,7 +26594,7 @@
         <v/>
       </c>
       <c r="H117" s="67" t="str">
-        <f aca="false">IF(A117="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A117,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A117="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A117,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A117,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A117,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A117,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I117" s="69" t="str">
@@ -26623,7 +26623,7 @@
         <v/>
       </c>
       <c r="H118" s="67" t="str">
-        <f aca="false">IF(A118="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A118,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A118="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A118,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A118,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A118,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A118,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I118" s="69" t="str">
@@ -26652,7 +26652,7 @@
         <v/>
       </c>
       <c r="H119" s="67" t="str">
-        <f aca="false">IF(A119="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A119,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A119="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A119,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A119,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A119,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A119,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I119" s="69" t="str">
@@ -26681,7 +26681,7 @@
         <v/>
       </c>
       <c r="H120" s="67" t="str">
-        <f aca="false">IF(A120="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A120,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A120="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A120,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A120,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A120,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A120,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I120" s="69" t="str">
@@ -26710,7 +26710,7 @@
         <v/>
       </c>
       <c r="H121" s="67" t="str">
-        <f aca="false">IF(A121="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A121,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A121="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A121,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A121,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A121,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A121,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I121" s="69" t="str">
@@ -26739,7 +26739,7 @@
         <v/>
       </c>
       <c r="H122" s="67" t="str">
-        <f aca="false">IF(A122="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A122,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A122="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A122,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A122,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A122,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A122,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I122" s="69" t="str">
@@ -26768,7 +26768,7 @@
         <v/>
       </c>
       <c r="H123" s="67" t="str">
-        <f aca="false">IF(A123="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A123,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A123="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A123,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A123,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A123,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A123,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I123" s="69" t="str">
@@ -26797,7 +26797,7 @@
         <v/>
       </c>
       <c r="H124" s="67" t="str">
-        <f aca="false">IF(A124="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A124,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A124="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A124,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A124,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A124,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A124,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I124" s="69" t="str">
@@ -26826,7 +26826,7 @@
         <v/>
       </c>
       <c r="H125" s="67" t="str">
-        <f aca="false">IF(A125="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A125,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A125="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A125,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A125,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A125,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A125,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I125" s="69" t="str">
@@ -26855,7 +26855,7 @@
         <v/>
       </c>
       <c r="H126" s="67" t="str">
-        <f aca="false">IF(A126="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A126,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A126="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A126,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A126,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A126,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A126,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I126" s="69" t="str">
@@ -26884,7 +26884,7 @@
         <v/>
       </c>
       <c r="H127" s="67" t="str">
-        <f aca="false">IF(A127="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A127,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A127="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A127,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A127,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A127,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A127,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I127" s="69" t="str">
@@ -26913,7 +26913,7 @@
         <v/>
       </c>
       <c r="H128" s="67" t="str">
-        <f aca="false">IF(A128="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A128,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A128="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A128,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A128,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A128,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A128,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I128" s="69" t="str">
@@ -26942,7 +26942,7 @@
         <v/>
       </c>
       <c r="H129" s="67" t="str">
-        <f aca="false">IF(A129="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A129,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A129="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A129,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A129,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A129,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A129,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I129" s="69" t="str">
@@ -26971,7 +26971,7 @@
         <v/>
       </c>
       <c r="H130" s="67" t="str">
-        <f aca="false">IF(A130="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A130,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A130="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A130,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A130,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A130,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A130,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I130" s="69" t="str">
@@ -27000,7 +27000,7 @@
         <v/>
       </c>
       <c r="H131" s="67" t="str">
-        <f aca="false">IF(A131="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A131,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A131="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A131,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A131,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A131,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A131,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I131" s="69" t="str">
@@ -27029,7 +27029,7 @@
         <v/>
       </c>
       <c r="H132" s="67" t="str">
-        <f aca="false">IF(A132="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A132,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A132="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A132,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A132,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A132,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A132,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I132" s="69" t="str">
@@ -27058,7 +27058,7 @@
         <v/>
       </c>
       <c r="H133" s="67" t="str">
-        <f aca="false">IF(A133="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A133,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A133="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A133,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A133,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A133,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A133,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I133" s="69" t="str">
@@ -27087,7 +27087,7 @@
         <v/>
       </c>
       <c r="H134" s="67" t="str">
-        <f aca="false">IF(A134="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A134,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A134="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A134,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A134,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A134,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A134,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I134" s="69" t="str">
@@ -27116,7 +27116,7 @@
         <v/>
       </c>
       <c r="H135" s="67" t="str">
-        <f aca="false">IF(A135="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A135,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A135="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A135,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A135,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A135,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A135,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I135" s="69" t="str">
@@ -27145,7 +27145,7 @@
         <v/>
       </c>
       <c r="H136" s="67" t="str">
-        <f aca="false">IF(A136="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A136,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A136="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A136,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A136,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A136,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A136,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I136" s="69" t="str">
@@ -27174,7 +27174,7 @@
         <v/>
       </c>
       <c r="H137" s="67" t="str">
-        <f aca="false">IF(A137="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A137,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A137="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A137,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A137,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A137,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A137,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I137" s="69" t="str">
@@ -27203,7 +27203,7 @@
         <v/>
       </c>
       <c r="H138" s="67" t="str">
-        <f aca="false">IF(A138="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A138,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A138="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A138,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A138,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A138,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A138,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I138" s="69" t="str">
@@ -27232,7 +27232,7 @@
         <v/>
       </c>
       <c r="H139" s="67" t="str">
-        <f aca="false">IF(A139="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A139,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A139="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A139,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A139,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A139,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A139,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I139" s="69" t="str">
@@ -27261,7 +27261,7 @@
         <v/>
       </c>
       <c r="H140" s="67" t="str">
-        <f aca="false">IF(A140="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A140,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A140="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A140,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A140,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A140,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A140,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I140" s="69" t="str">
@@ -27290,7 +27290,7 @@
         <v/>
       </c>
       <c r="H141" s="67" t="str">
-        <f aca="false">IF(A141="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A141,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A141="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A141,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A141,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A141,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A141,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I141" s="69" t="str">
@@ -27319,7 +27319,7 @@
         <v/>
       </c>
       <c r="H142" s="67" t="str">
-        <f aca="false">IF(A142="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A142,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A142="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A142,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A142,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A142,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A142,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I142" s="69" t="str">
@@ -27348,7 +27348,7 @@
         <v/>
       </c>
       <c r="H143" s="67" t="str">
-        <f aca="false">IF(A143="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A143,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A143="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A143,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A143,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A143,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A143,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I143" s="69" t="str">
@@ -27377,7 +27377,7 @@
         <v/>
       </c>
       <c r="H144" s="67" t="str">
-        <f aca="false">IF(A144="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A144,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A144="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A144,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A144,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A144,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A144,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I144" s="69" t="str">
@@ -27406,7 +27406,7 @@
         <v/>
       </c>
       <c r="H145" s="67" t="str">
-        <f aca="false">IF(A145="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A145,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A145="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A145,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A145,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A145,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A145,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I145" s="69" t="str">
@@ -27435,7 +27435,7 @@
         <v/>
       </c>
       <c r="H146" s="67" t="str">
-        <f aca="false">IF(A146="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A146,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A146="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A146,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A146,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A146,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A146,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I146" s="69" t="str">
@@ -27464,7 +27464,7 @@
         <v/>
       </c>
       <c r="H147" s="67" t="str">
-        <f aca="false">IF(A147="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A147,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A147="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A147,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A147,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A147,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A147,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I147" s="69" t="str">
@@ -27493,7 +27493,7 @@
         <v/>
       </c>
       <c r="H148" s="67" t="str">
-        <f aca="false">IF(A148="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A148,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A148="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A148,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A148,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A148,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A148,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I148" s="69" t="str">
@@ -27522,7 +27522,7 @@
         <v/>
       </c>
       <c r="H149" s="67" t="str">
-        <f aca="false">IF(A149="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A149,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A149="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A149,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A149,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A149,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A149,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I149" s="69" t="str">
@@ -27551,7 +27551,7 @@
         <v/>
       </c>
       <c r="H150" s="67" t="str">
-        <f aca="false">IF(A150="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A150,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A150="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A150,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A150,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A150,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A150,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I150" s="69" t="str">
@@ -27580,7 +27580,7 @@
         <v/>
       </c>
       <c r="H151" s="67" t="str">
-        <f aca="false">IF(A151="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A151,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A151="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A151,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A151,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A151,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A151,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I151" s="69" t="str">
@@ -27609,7 +27609,7 @@
         <v/>
       </c>
       <c r="H152" s="67" t="str">
-        <f aca="false">IF(A152="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A152,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A152="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A152,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A152,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A152,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A152,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I152" s="69" t="str">
@@ -27638,7 +27638,7 @@
         <v/>
       </c>
       <c r="H153" s="67" t="str">
-        <f aca="false">IF(A153="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A153,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A153="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A153,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A153,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A153,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A153,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I153" s="69" t="str">
@@ -27667,7 +27667,7 @@
         <v/>
       </c>
       <c r="H154" s="67" t="str">
-        <f aca="false">IF(A154="","",SUMPRODUCT(COUNTIFS('RFQ Log'!$C$5:$C$304,A154,'RFQ Log'!$R$5:$R$304,{"Won","Ordered","Shipped","Paid"})))</f>
+        <f aca="false">IF(A154="","",COUNTIFS('RFQ Log'!$C$5:$C$304,A154,'RFQ Log'!$R$5:$R$304,"Won")+COUNTIFS('RFQ Log'!$C$5:$C$304,A154,'RFQ Log'!$R$5:$R$304,"Ordered")+COUNTIFS('RFQ Log'!$C$5:$C$304,A154,'RFQ Log'!$R$5:$R$304,"Shipped")+COUNTIFS('RFQ Log'!$C$5:$C$304,A154,'RFQ Log'!$R$5:$R$304,"Paid"))</f>
         <v/>
       </c>
       <c r="I154" s="69" t="str">

</xml_diff>